<commit_message>
Update reports 2026-09-09 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-09.xlsx
+++ b/gex_pivot_levels_2026-09-09.xlsx
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$7.20M</t>
+          <t>-$7.83M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$10.98M</t>
+          <t>+$11.94M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>-$17.31M</t>
+          <t>-$18.82M</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>+$18.99M</t>
+          <t>+$20.64M</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>-$1.59M</t>
+          <t>-$1.73M</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>+$13.17M</t>
+          <t>+$14.33M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -771,12 +771,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-$10.04M</t>
+          <t>-$10.77M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$24.05M</t>
+          <t>+$25.79M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>-$10.31M</t>
+          <t>-$10.95M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$12.88M</t>
+          <t>+$13.68M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>-$3.74M</t>
+          <t>-$3.90M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$16.46M</t>
+          <t>+$17.16M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -965,12 +965,12 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>-$26.17M</t>
+          <t>-$26.97M</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>+$43.92M</t>
+          <t>+$45.26M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1031,12 +1031,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$2.89M</t>
+          <t>+$2.81M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$19.41M</t>
+          <t>+$18.86M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1064,12 +1064,12 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>-$14.76M</t>
+          <t>-$14.04M</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>+$50.28M</t>
+          <t>+$47.84M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>+$17.48M</t>
+          <t>+$15.49M</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>+$20.36M</t>
+          <t>+$18.04M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1196,12 +1196,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>+$5.02M</t>
+          <t>+$4.52M</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>+$8.36M</t>
+          <t>+$7.52M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -3165,12 +3165,12 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>-$14.76M</t>
+          <t>-$14.04M</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>+$50.28M</t>
+          <t>+$47.84M</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -3203,12 +3203,12 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>-$26.17M</t>
+          <t>-$26.97M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>+$43.92M</t>
+          <t>+$45.26M</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -3317,12 +3317,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>-$10.04M</t>
+          <t>-$10.77M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>+$24.05M</t>
+          <t>+$25.79M</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -3373,28 +3373,28 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>29747.27</v>
+        <v>7641.48</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>722</v>
+        <v>7630</v>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>+$18.66M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-$18.82M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>+$20.48M</t>
+          <t>+$20.64M</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3404,121 +3404,121 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>29747.27</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>722</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>+$18.66M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>+$20.48M</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
-        <v>7741.48</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>7730</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="B10" s="5" t="n">
+        <v>7625.29</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>760</v>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>-$12.66M</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>+$18.89M</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>7701.48</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>7690</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>+$17.48M</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>+$20.36M</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>+$2.81M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>+$18.86M</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>7701.48</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>7690</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>+$2.89M</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>+$19.41M</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>7641.48</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>7630</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>-$17.31M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>+$18.99M</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3529,10 +3529,10 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7625.29</v>
+        <v>7675.38</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
@@ -3541,12 +3541,12 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>-$12.66M</t>
+          <t>-$1.47M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>+$18.89M</t>
+          <t>+$18.62M</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3567,24 +3567,24 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7675.38</v>
+        <v>7741.48</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>765</v>
+        <v>7730</v>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>-$1.47M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>+$15.49M</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>+$18.62M</t>
+          <t>+$18.04M</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -3599,78 +3599,78 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>7681.48</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>7670</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>-$3.90M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>+$17.16M</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B15" s="5" t="n">
         <v>2967.7</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C15" s="5" t="n">
         <v>295</v>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>-$1.92M</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>+$17.16M</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>7681.48</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>7670</v>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>-$3.74M</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>+$16.46M</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3753,24 +3753,24 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>7665.36</v>
+        <v>7651.48</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>764</v>
+        <v>7640</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>-$3.91M</t>
+          <t>-$1.73M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>+$13.80M</t>
+          <t>+$14.33M</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -3791,24 +3791,24 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>7651.48</v>
+        <v>7665.36</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>7640</v>
+        <v>764</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>-$1.59M</t>
+          <t>-$3.91M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$13.17M</t>
+          <t>+$13.80M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3841,12 +3841,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>-$10.31M</t>
+          <t>-$10.95M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$12.88M</t>
+          <t>+$13.68M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -3937,148 +3937,148 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>7611.48</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>7600</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>-$7.83M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>+$11.94M</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
+      <c r="B24" s="5" t="n">
         <v>4538.48</v>
       </c>
-      <c r="C23" s="5" t="n">
+      <c r="C24" s="5" t="n">
         <v>101</v>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>+$10.98M</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>+$11.25M</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>4673.29</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>104</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>+$7.76M</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>+$7.84M</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
-        <v>7611.48</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="B26" s="2" t="n">
+        <v>7761.48</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>-$7.20M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>+$10.98M</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>+$4.52M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$7.52M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>7761.48</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>+$5.02M</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>+$8.36M</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>4673.29</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>104</v>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>+$7.76M</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>+$7.84M</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">

</xml_diff>